<commit_message>
Direct Write Excel for QC-03 Day 5
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-03.xlsx
+++ b/FM-MN-07_QC-03.xlsx
@@ -1742,7 +1742,11 @@
       <c r="D6" s="26" t="n"/>
       <c r="E6" s="26" t="n"/>
       <c r="F6" s="26" t="n"/>
-      <c r="G6" s="26" t="n"/>
+      <c r="G6" s="26" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="H6" s="26" t="n"/>
       <c r="I6" s="26" t="n"/>
       <c r="J6" s="26" t="n"/>
@@ -1791,7 +1795,11 @@
       <c r="D7" s="26" t="n"/>
       <c r="E7" s="26" t="n"/>
       <c r="F7" s="26" t="n"/>
-      <c r="G7" s="26" t="n"/>
+      <c r="G7" s="26" t="inlineStr">
+        <is>
+          <t>⨂</t>
+        </is>
+      </c>
       <c r="H7" s="26" t="n"/>
       <c r="I7" s="26" t="n"/>
       <c r="J7" s="26" t="n"/>
@@ -1840,7 +1848,11 @@
       <c r="D8" s="26" t="n"/>
       <c r="E8" s="26" t="n"/>
       <c r="F8" s="26" t="n"/>
-      <c r="G8" s="26" t="n"/>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H8" s="26" t="n"/>
       <c r="I8" s="26" t="n"/>
       <c r="J8" s="26" t="n"/>
@@ -1889,7 +1901,11 @@
       <c r="D9" s="26" t="n"/>
       <c r="E9" s="26" t="n"/>
       <c r="F9" s="26" t="n"/>
-      <c r="G9" s="26" t="n"/>
+      <c r="G9" s="26" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
       <c r="H9" s="26" t="n"/>
       <c r="I9" s="26" t="n"/>
       <c r="J9" s="26" t="n"/>
@@ -1938,7 +1954,11 @@
       <c r="D10" s="26" t="n"/>
       <c r="E10" s="26" t="n"/>
       <c r="F10" s="26" t="n"/>
-      <c r="G10" s="26" t="n"/>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>⨂</t>
+        </is>
+      </c>
       <c r="H10" s="26" t="n"/>
       <c r="I10" s="26" t="n"/>
       <c r="J10" s="26" t="n"/>
@@ -1981,7 +2001,11 @@
       <c r="D11" s="38" t="n"/>
       <c r="E11" s="38" t="n"/>
       <c r="F11" s="38" t="n"/>
-      <c r="G11" s="38" t="n"/>
+      <c r="G11" s="40" t="inlineStr">
+        <is>
+          <t>เค</t>
+        </is>
+      </c>
       <c r="H11" s="38" t="n"/>
       <c r="I11" s="38" t="n"/>
       <c r="J11" s="38" t="n"/>
@@ -2172,8 +2196,8 @@
     <mergeCell ref="H11:H12"/>
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AG11:AG12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>

</xml_diff>

<commit_message>
Direct Write Excel for QC-03 Day 6
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-03.xlsx
+++ b/FM-MN-07_QC-03.xlsx
@@ -1718,7 +1718,11 @@
       <c r="E6" s="10" t="inlineStr"/>
       <c r="F6" s="10" t="inlineStr"/>
       <c r="G6" s="10" t="inlineStr"/>
-      <c r="H6" s="10" t="inlineStr"/>
+      <c r="H6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I6" s="10" t="inlineStr"/>
       <c r="J6" s="10" t="inlineStr"/>
       <c r="K6" s="10" t="inlineStr"/>
@@ -1759,7 +1763,11 @@
       <c r="E7" s="10" t="inlineStr"/>
       <c r="F7" s="10" t="inlineStr"/>
       <c r="G7" s="10" t="inlineStr"/>
-      <c r="H7" s="10" t="inlineStr"/>
+      <c r="H7" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I7" s="10" t="inlineStr"/>
       <c r="J7" s="10" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
@@ -1800,7 +1808,11 @@
       <c r="E8" s="10" t="inlineStr"/>
       <c r="F8" s="10" t="inlineStr"/>
       <c r="G8" s="10" t="inlineStr"/>
-      <c r="H8" s="10" t="inlineStr"/>
+      <c r="H8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I8" s="10" t="inlineStr"/>
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
@@ -1841,7 +1853,11 @@
       <c r="E9" s="10" t="inlineStr"/>
       <c r="F9" s="10" t="inlineStr"/>
       <c r="G9" s="10" t="inlineStr"/>
-      <c r="H9" s="10" t="inlineStr"/>
+      <c r="H9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I9" s="10" t="inlineStr"/>
       <c r="J9" s="10" t="inlineStr"/>
       <c r="K9" s="10" t="inlineStr"/>
@@ -1882,7 +1898,11 @@
       <c r="E10" s="10" t="inlineStr"/>
       <c r="F10" s="10" t="inlineStr"/>
       <c r="G10" s="10" t="inlineStr"/>
-      <c r="H10" s="10" t="inlineStr"/>
+      <c r="H10" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="I10" s="10" t="inlineStr"/>
       <c r="J10" s="10" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
@@ -1917,7 +1937,11 @@
       <c r="E11" s="20" t="inlineStr"/>
       <c r="F11" s="20" t="inlineStr"/>
       <c r="G11" s="20" t="inlineStr"/>
-      <c r="H11" s="20" t="inlineStr"/>
+      <c r="H11" s="31" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="I11" s="20" t="inlineStr"/>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
@@ -2100,8 +2124,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-03 Day 7
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-03.xlsx
+++ b/FM-MN-07_QC-03.xlsx
@@ -1726,7 +1726,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I6" s="10" t="inlineStr"/>
+      <c r="I6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J6" s="10" t="inlineStr"/>
       <c r="K6" s="10" t="inlineStr"/>
       <c r="L6" s="10" t="inlineStr"/>
@@ -1771,7 +1775,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I7" s="10" t="inlineStr"/>
+      <c r="I7" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J7" s="10" t="inlineStr"/>
       <c r="K7" s="10" t="inlineStr"/>
       <c r="L7" s="10" t="inlineStr"/>
@@ -1816,7 +1824,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I8" s="10" t="inlineStr"/>
+      <c r="I8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J8" s="10" t="inlineStr"/>
       <c r="K8" s="10" t="inlineStr"/>
       <c r="L8" s="10" t="inlineStr"/>
@@ -1861,7 +1873,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I9" s="10" t="inlineStr"/>
+      <c r="I9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J9" s="10" t="inlineStr"/>
       <c r="K9" s="10" t="inlineStr"/>
       <c r="L9" s="10" t="inlineStr"/>
@@ -1906,7 +1922,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="I10" s="10" t="inlineStr"/>
+      <c r="I10" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="J10" s="10" t="inlineStr"/>
       <c r="K10" s="10" t="inlineStr"/>
       <c r="L10" s="10" t="inlineStr"/>
@@ -1945,7 +1965,11 @@
           <t>สัมพันธ์ รักวิถี</t>
         </is>
       </c>
-      <c r="I11" s="20" t="inlineStr"/>
+      <c r="I11" s="31" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="J11" s="20" t="inlineStr"/>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
@@ -2131,8 +2155,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-03 Day 8
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-03.xlsx
+++ b/FM-MN-07_QC-03.xlsx
@@ -1731,7 +1731,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J6" s="10" t="inlineStr"/>
+      <c r="J6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K6" s="10" t="inlineStr"/>
       <c r="L6" s="10" t="inlineStr"/>
       <c r="M6" s="10" t="inlineStr"/>
@@ -1780,7 +1784,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J7" s="10" t="inlineStr"/>
+      <c r="J7" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K7" s="10" t="inlineStr"/>
       <c r="L7" s="10" t="inlineStr"/>
       <c r="M7" s="10" t="inlineStr"/>
@@ -1829,7 +1837,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J8" s="10" t="inlineStr"/>
+      <c r="J8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K8" s="10" t="inlineStr"/>
       <c r="L8" s="10" t="inlineStr"/>
       <c r="M8" s="10" t="inlineStr"/>
@@ -1878,7 +1890,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J9" s="10" t="inlineStr"/>
+      <c r="J9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K9" s="10" t="inlineStr"/>
       <c r="L9" s="10" t="inlineStr"/>
       <c r="M9" s="10" t="inlineStr"/>
@@ -1927,7 +1943,11 @@
           <t>/</t>
         </is>
       </c>
-      <c r="J10" s="10" t="inlineStr"/>
+      <c r="J10" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="K10" s="10" t="inlineStr"/>
       <c r="L10" s="10" t="inlineStr"/>
       <c r="M10" s="10" t="inlineStr"/>
@@ -1970,7 +1990,11 @@
           <t>สัมพันธ์ รักวิถี</t>
         </is>
       </c>
-      <c r="J11" s="20" t="inlineStr"/>
+      <c r="J11" s="31" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="K11" s="20" t="inlineStr"/>
       <c r="L11" s="20" t="inlineStr"/>
       <c r="M11" s="20" t="inlineStr"/>
@@ -2155,8 +2179,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="P11:P12"/>
     <mergeCell ref="B16:AG16"/>
-    <mergeCell ref="P11:P12"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>

<commit_message>
Safe Direct Write Excel for QC-03 Day 10
</commit_message>
<xml_diff>
--- a/FM-MN-07_QC-03.xlsx
+++ b/FM-MN-07_QC-03.xlsx
@@ -1737,7 +1737,11 @@
         </is>
       </c>
       <c r="K6" s="10" t="inlineStr"/>
-      <c r="L6" s="10" t="inlineStr"/>
+      <c r="L6" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M6" s="10" t="inlineStr"/>
       <c r="N6" s="10" t="inlineStr"/>
       <c r="O6" s="10" t="inlineStr"/>
@@ -1790,7 +1794,11 @@
         </is>
       </c>
       <c r="K7" s="10" t="inlineStr"/>
-      <c r="L7" s="10" t="inlineStr"/>
+      <c r="L7" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M7" s="10" t="inlineStr"/>
       <c r="N7" s="10" t="inlineStr"/>
       <c r="O7" s="10" t="inlineStr"/>
@@ -1843,7 +1851,11 @@
         </is>
       </c>
       <c r="K8" s="10" t="inlineStr"/>
-      <c r="L8" s="10" t="inlineStr"/>
+      <c r="L8" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M8" s="10" t="inlineStr"/>
       <c r="N8" s="10" t="inlineStr"/>
       <c r="O8" s="10" t="inlineStr"/>
@@ -1896,7 +1908,11 @@
         </is>
       </c>
       <c r="K9" s="10" t="inlineStr"/>
-      <c r="L9" s="10" t="inlineStr"/>
+      <c r="L9" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M9" s="10" t="inlineStr"/>
       <c r="N9" s="10" t="inlineStr"/>
       <c r="O9" s="10" t="inlineStr"/>
@@ -1949,7 +1965,11 @@
         </is>
       </c>
       <c r="K10" s="10" t="inlineStr"/>
-      <c r="L10" s="10" t="inlineStr"/>
+      <c r="L10" s="10" t="inlineStr">
+        <is>
+          <t>/</t>
+        </is>
+      </c>
       <c r="M10" s="10" t="inlineStr"/>
       <c r="N10" s="10" t="inlineStr"/>
       <c r="O10" s="10" t="inlineStr"/>
@@ -1996,7 +2016,11 @@
         </is>
       </c>
       <c r="K11" s="20" t="inlineStr"/>
-      <c r="L11" s="20" t="inlineStr"/>
+      <c r="L11" s="31" t="inlineStr">
+        <is>
+          <t>สัมพันธ์ รักวิถี</t>
+        </is>
+      </c>
       <c r="M11" s="20" t="inlineStr"/>
       <c r="N11" s="20" t="inlineStr"/>
       <c r="O11" s="20" t="inlineStr"/>
@@ -2179,8 +2203,8 @@
     <mergeCell ref="Y11:Y12"/>
     <mergeCell ref="J11:J12"/>
     <mergeCell ref="AG11:AG12"/>
+    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="P11:P12"/>
-    <mergeCell ref="B16:AG16"/>
     <mergeCell ref="AB2:AG2"/>
     <mergeCell ref="AC18:AG18"/>
     <mergeCell ref="K11:K12"/>

</xml_diff>